<commit_message>
Ignore .claude/ local settings and update 5-1.xlsx
</commit_message>
<xml_diff>
--- a/data_clean/5-1.xlsx
+++ b/data_clean/5-1.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10814"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F9EBC82-46BF-FF4A-9BF8-F5E89E0B8BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-12" yWindow="-12" windowWidth="19416" windowHeight="5832" tabRatio="723"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ｖ１中分類 (実数ウエイト)" sheetId="24" r:id="rId1"/>
@@ -640,17 +641,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="176" formatCode="0_ "/>
-    <numFmt numFmtId="177" formatCode="#\ ###\ ###\ ##0"/>
-    <numFmt numFmtId="178" formatCode="###\ ###\ ##0"/>
+    <numFmt numFmtId="164" formatCode="0_ "/>
+    <numFmt numFmtId="165" formatCode="#\ ###\ ###\ ##0"/>
+    <numFmt numFmtId="166" formatCode="###\ ###\ ##0"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="ＭＳ Ｐゴシック"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -999,26 +1000,24 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="5" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="5" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
@@ -1027,13 +1026,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="6" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
@@ -1042,13 +1041,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="4" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1072,10 +1071,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1092,154 +1091,154 @@
     </xf>
   </cellXfs>
   <cellStyles count="148">
-    <cellStyle name="パーセント 2" xfId="1"/>
-    <cellStyle name="桁区切り 2" xfId="2"/>
-    <cellStyle name="桁区切り 3" xfId="3"/>
-    <cellStyle name="桁区切り 4" xfId="4"/>
-    <cellStyle name="標準" xfId="0" builtinId="0"/>
-    <cellStyle name="標準 2" xfId="5"/>
-    <cellStyle name="標準 2 10" xfId="6"/>
-    <cellStyle name="標準 2 100" xfId="7"/>
-    <cellStyle name="標準 2 101" xfId="8"/>
-    <cellStyle name="標準 2 102" xfId="9"/>
-    <cellStyle name="標準 2 103" xfId="10"/>
-    <cellStyle name="標準 2 104" xfId="11"/>
-    <cellStyle name="標準 2 105" xfId="12"/>
-    <cellStyle name="標準 2 106" xfId="13"/>
-    <cellStyle name="標準 2 107" xfId="14"/>
-    <cellStyle name="標準 2 108" xfId="15"/>
-    <cellStyle name="標準 2 109" xfId="16"/>
-    <cellStyle name="標準 2 11" xfId="17"/>
-    <cellStyle name="標準 2 110" xfId="18"/>
-    <cellStyle name="標準 2 111" xfId="19"/>
-    <cellStyle name="標準 2 112" xfId="20"/>
-    <cellStyle name="標準 2 113" xfId="21"/>
-    <cellStyle name="標準 2 114" xfId="22"/>
-    <cellStyle name="標準 2 115" xfId="23"/>
-    <cellStyle name="標準 2 116" xfId="24"/>
-    <cellStyle name="標準 2 117" xfId="25"/>
-    <cellStyle name="標準 2 118" xfId="26"/>
-    <cellStyle name="標準 2 119" xfId="27"/>
-    <cellStyle name="標準 2 12" xfId="28"/>
-    <cellStyle name="標準 2 120" xfId="29"/>
-    <cellStyle name="標準 2 121" xfId="30"/>
-    <cellStyle name="標準 2 122" xfId="31"/>
-    <cellStyle name="標準 2 123" xfId="32"/>
-    <cellStyle name="標準 2 124" xfId="33"/>
-    <cellStyle name="標準 2 125" xfId="34"/>
-    <cellStyle name="標準 2 126" xfId="35"/>
-    <cellStyle name="標準 2 127" xfId="36"/>
-    <cellStyle name="標準 2 128" xfId="37"/>
-    <cellStyle name="標準 2 129" xfId="38"/>
-    <cellStyle name="標準 2 13" xfId="39"/>
-    <cellStyle name="標準 2 130" xfId="40"/>
-    <cellStyle name="標準 2 131" xfId="41"/>
-    <cellStyle name="標準 2 132" xfId="42"/>
-    <cellStyle name="標準 2 133" xfId="43"/>
-    <cellStyle name="標準 2 134" xfId="44"/>
-    <cellStyle name="標準 2 135" xfId="45"/>
-    <cellStyle name="標準 2 136" xfId="46"/>
-    <cellStyle name="標準 2 137" xfId="47"/>
-    <cellStyle name="標準 2 138" xfId="48"/>
-    <cellStyle name="標準 2 139" xfId="49"/>
-    <cellStyle name="標準 2 14" xfId="50"/>
-    <cellStyle name="標準 2 15" xfId="51"/>
-    <cellStyle name="標準 2 16" xfId="52"/>
-    <cellStyle name="標準 2 17" xfId="53"/>
-    <cellStyle name="標準 2 18" xfId="54"/>
-    <cellStyle name="標準 2 19" xfId="55"/>
-    <cellStyle name="標準 2 2" xfId="56"/>
-    <cellStyle name="標準 2 20" xfId="57"/>
-    <cellStyle name="標準 2 21" xfId="58"/>
-    <cellStyle name="標準 2 22" xfId="59"/>
-    <cellStyle name="標準 2 23" xfId="60"/>
-    <cellStyle name="標準 2 24" xfId="61"/>
-    <cellStyle name="標準 2 25" xfId="62"/>
-    <cellStyle name="標準 2 26" xfId="63"/>
-    <cellStyle name="標準 2 27" xfId="64"/>
-    <cellStyle name="標準 2 28" xfId="65"/>
-    <cellStyle name="標準 2 29" xfId="66"/>
-    <cellStyle name="標準 2 3" xfId="67"/>
-    <cellStyle name="標準 2 30" xfId="68"/>
-    <cellStyle name="標準 2 31" xfId="69"/>
-    <cellStyle name="標準 2 32" xfId="70"/>
-    <cellStyle name="標準 2 33" xfId="71"/>
-    <cellStyle name="標準 2 34" xfId="72"/>
-    <cellStyle name="標準 2 35" xfId="73"/>
-    <cellStyle name="標準 2 36" xfId="74"/>
-    <cellStyle name="標準 2 37" xfId="75"/>
-    <cellStyle name="標準 2 38" xfId="76"/>
-    <cellStyle name="標準 2 39" xfId="77"/>
-    <cellStyle name="標準 2 4" xfId="78"/>
-    <cellStyle name="標準 2 40" xfId="79"/>
-    <cellStyle name="標準 2 41" xfId="80"/>
-    <cellStyle name="標準 2 42" xfId="81"/>
-    <cellStyle name="標準 2 43" xfId="82"/>
-    <cellStyle name="標準 2 44" xfId="83"/>
-    <cellStyle name="標準 2 45" xfId="84"/>
-    <cellStyle name="標準 2 46" xfId="85"/>
-    <cellStyle name="標準 2 47" xfId="86"/>
-    <cellStyle name="標準 2 48" xfId="87"/>
-    <cellStyle name="標準 2 49" xfId="88"/>
-    <cellStyle name="標準 2 5" xfId="89"/>
-    <cellStyle name="標準 2 50" xfId="90"/>
-    <cellStyle name="標準 2 51" xfId="91"/>
-    <cellStyle name="標準 2 52" xfId="92"/>
-    <cellStyle name="標準 2 53" xfId="93"/>
-    <cellStyle name="標準 2 54" xfId="94"/>
-    <cellStyle name="標準 2 55" xfId="95"/>
-    <cellStyle name="標準 2 56" xfId="96"/>
-    <cellStyle name="標準 2 57" xfId="97"/>
-    <cellStyle name="標準 2 58" xfId="98"/>
-    <cellStyle name="標準 2 59" xfId="99"/>
-    <cellStyle name="標準 2 6" xfId="100"/>
-    <cellStyle name="標準 2 60" xfId="101"/>
-    <cellStyle name="標準 2 61" xfId="102"/>
-    <cellStyle name="標準 2 62" xfId="103"/>
-    <cellStyle name="標準 2 63" xfId="104"/>
-    <cellStyle name="標準 2 64" xfId="105"/>
-    <cellStyle name="標準 2 65" xfId="106"/>
-    <cellStyle name="標準 2 66" xfId="107"/>
-    <cellStyle name="標準 2 67" xfId="108"/>
-    <cellStyle name="標準 2 68" xfId="109"/>
-    <cellStyle name="標準 2 69" xfId="110"/>
-    <cellStyle name="標準 2 7" xfId="111"/>
-    <cellStyle name="標準 2 70" xfId="112"/>
-    <cellStyle name="標準 2 71" xfId="113"/>
-    <cellStyle name="標準 2 72" xfId="114"/>
-    <cellStyle name="標準 2 73" xfId="115"/>
-    <cellStyle name="標準 2 74" xfId="116"/>
-    <cellStyle name="標準 2 75" xfId="117"/>
-    <cellStyle name="標準 2 76" xfId="118"/>
-    <cellStyle name="標準 2 77" xfId="119"/>
-    <cellStyle name="標準 2 78" xfId="120"/>
-    <cellStyle name="標準 2 79" xfId="121"/>
-    <cellStyle name="標準 2 8" xfId="122"/>
-    <cellStyle name="標準 2 80" xfId="123"/>
-    <cellStyle name="標準 2 81" xfId="124"/>
-    <cellStyle name="標準 2 82" xfId="125"/>
-    <cellStyle name="標準 2 83" xfId="126"/>
-    <cellStyle name="標準 2 84" xfId="127"/>
-    <cellStyle name="標準 2 85" xfId="128"/>
-    <cellStyle name="標準 2 86" xfId="129"/>
-    <cellStyle name="標準 2 87" xfId="130"/>
-    <cellStyle name="標準 2 88" xfId="131"/>
-    <cellStyle name="標準 2 89" xfId="132"/>
-    <cellStyle name="標準 2 9" xfId="133"/>
-    <cellStyle name="標準 2 90" xfId="134"/>
-    <cellStyle name="標準 2 91" xfId="135"/>
-    <cellStyle name="標準 2 92" xfId="136"/>
-    <cellStyle name="標準 2 93" xfId="137"/>
-    <cellStyle name="標準 2 94" xfId="138"/>
-    <cellStyle name="標準 2 95" xfId="139"/>
-    <cellStyle name="標準 2 96" xfId="140"/>
-    <cellStyle name="標準 2 97" xfId="141"/>
-    <cellStyle name="標準 2 98" xfId="142"/>
-    <cellStyle name="標準 2 99" xfId="143"/>
-    <cellStyle name="標準 3" xfId="144"/>
-    <cellStyle name="標準 4" xfId="145"/>
-    <cellStyle name="標準 5" xfId="146"/>
-    <cellStyle name="標準 6" xfId="147"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="パーセント 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="桁区切り 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="桁区切り 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="桁区切り 4" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="標準 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="標準 2 10" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="標準 2 100" xfId="7" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="標準 2 101" xfId="8" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="標準 2 102" xfId="9" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="標準 2 103" xfId="10" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="標準 2 104" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="標準 2 105" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="標準 2 106" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="標準 2 107" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="標準 2 108" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="標準 2 109" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="標準 2 11" xfId="17" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="標準 2 110" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="標準 2 111" xfId="19" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="標準 2 112" xfId="20" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="標準 2 113" xfId="21" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="標準 2 114" xfId="22" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="標準 2 115" xfId="23" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="標準 2 116" xfId="24" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="標準 2 117" xfId="25" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="標準 2 118" xfId="26" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="標準 2 119" xfId="27" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="標準 2 12" xfId="28" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="標準 2 120" xfId="29" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="標準 2 121" xfId="30" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="標準 2 122" xfId="31" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="標準 2 123" xfId="32" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="標準 2 124" xfId="33" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="標準 2 125" xfId="34" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="標準 2 126" xfId="35" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="標準 2 127" xfId="36" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="標準 2 128" xfId="37" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="標準 2 129" xfId="38" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="標準 2 13" xfId="39" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
+    <cellStyle name="標準 2 130" xfId="40" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
+    <cellStyle name="標準 2 131" xfId="41" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
+    <cellStyle name="標準 2 132" xfId="42" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
+    <cellStyle name="標準 2 133" xfId="43" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
+    <cellStyle name="標準 2 134" xfId="44" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
+    <cellStyle name="標準 2 135" xfId="45" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
+    <cellStyle name="標準 2 136" xfId="46" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
+    <cellStyle name="標準 2 137" xfId="47" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
+    <cellStyle name="標準 2 138" xfId="48" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
+    <cellStyle name="標準 2 139" xfId="49" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="標準 2 14" xfId="50" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
+    <cellStyle name="標準 2 15" xfId="51" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
+    <cellStyle name="標準 2 16" xfId="52" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
+    <cellStyle name="標準 2 17" xfId="53" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
+    <cellStyle name="標準 2 18" xfId="54" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
+    <cellStyle name="標準 2 19" xfId="55" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
+    <cellStyle name="標準 2 2" xfId="56" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
+    <cellStyle name="標準 2 20" xfId="57" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
+    <cellStyle name="標準 2 21" xfId="58" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
+    <cellStyle name="標準 2 22" xfId="59" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
+    <cellStyle name="標準 2 23" xfId="60" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
+    <cellStyle name="標準 2 24" xfId="61" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
+    <cellStyle name="標準 2 25" xfId="62" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
+    <cellStyle name="標準 2 26" xfId="63" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
+    <cellStyle name="標準 2 27" xfId="64" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
+    <cellStyle name="標準 2 28" xfId="65" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
+    <cellStyle name="標準 2 29" xfId="66" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
+    <cellStyle name="標準 2 3" xfId="67" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
+    <cellStyle name="標準 2 30" xfId="68" xr:uid="{00000000-0005-0000-0000-000044000000}"/>
+    <cellStyle name="標準 2 31" xfId="69" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
+    <cellStyle name="標準 2 32" xfId="70" xr:uid="{00000000-0005-0000-0000-000046000000}"/>
+    <cellStyle name="標準 2 33" xfId="71" xr:uid="{00000000-0005-0000-0000-000047000000}"/>
+    <cellStyle name="標準 2 34" xfId="72" xr:uid="{00000000-0005-0000-0000-000048000000}"/>
+    <cellStyle name="標準 2 35" xfId="73" xr:uid="{00000000-0005-0000-0000-000049000000}"/>
+    <cellStyle name="標準 2 36" xfId="74" xr:uid="{00000000-0005-0000-0000-00004A000000}"/>
+    <cellStyle name="標準 2 37" xfId="75" xr:uid="{00000000-0005-0000-0000-00004B000000}"/>
+    <cellStyle name="標準 2 38" xfId="76" xr:uid="{00000000-0005-0000-0000-00004C000000}"/>
+    <cellStyle name="標準 2 39" xfId="77" xr:uid="{00000000-0005-0000-0000-00004D000000}"/>
+    <cellStyle name="標準 2 4" xfId="78" xr:uid="{00000000-0005-0000-0000-00004E000000}"/>
+    <cellStyle name="標準 2 40" xfId="79" xr:uid="{00000000-0005-0000-0000-00004F000000}"/>
+    <cellStyle name="標準 2 41" xfId="80" xr:uid="{00000000-0005-0000-0000-000050000000}"/>
+    <cellStyle name="標準 2 42" xfId="81" xr:uid="{00000000-0005-0000-0000-000051000000}"/>
+    <cellStyle name="標準 2 43" xfId="82" xr:uid="{00000000-0005-0000-0000-000052000000}"/>
+    <cellStyle name="標準 2 44" xfId="83" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
+    <cellStyle name="標準 2 45" xfId="84" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
+    <cellStyle name="標準 2 46" xfId="85" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
+    <cellStyle name="標準 2 47" xfId="86" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
+    <cellStyle name="標準 2 48" xfId="87" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
+    <cellStyle name="標準 2 49" xfId="88" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
+    <cellStyle name="標準 2 5" xfId="89" xr:uid="{00000000-0005-0000-0000-000059000000}"/>
+    <cellStyle name="標準 2 50" xfId="90" xr:uid="{00000000-0005-0000-0000-00005A000000}"/>
+    <cellStyle name="標準 2 51" xfId="91" xr:uid="{00000000-0005-0000-0000-00005B000000}"/>
+    <cellStyle name="標準 2 52" xfId="92" xr:uid="{00000000-0005-0000-0000-00005C000000}"/>
+    <cellStyle name="標準 2 53" xfId="93" xr:uid="{00000000-0005-0000-0000-00005D000000}"/>
+    <cellStyle name="標準 2 54" xfId="94" xr:uid="{00000000-0005-0000-0000-00005E000000}"/>
+    <cellStyle name="標準 2 55" xfId="95" xr:uid="{00000000-0005-0000-0000-00005F000000}"/>
+    <cellStyle name="標準 2 56" xfId="96" xr:uid="{00000000-0005-0000-0000-000060000000}"/>
+    <cellStyle name="標準 2 57" xfId="97" xr:uid="{00000000-0005-0000-0000-000061000000}"/>
+    <cellStyle name="標準 2 58" xfId="98" xr:uid="{00000000-0005-0000-0000-000062000000}"/>
+    <cellStyle name="標準 2 59" xfId="99" xr:uid="{00000000-0005-0000-0000-000063000000}"/>
+    <cellStyle name="標準 2 6" xfId="100" xr:uid="{00000000-0005-0000-0000-000064000000}"/>
+    <cellStyle name="標準 2 60" xfId="101" xr:uid="{00000000-0005-0000-0000-000065000000}"/>
+    <cellStyle name="標準 2 61" xfId="102" xr:uid="{00000000-0005-0000-0000-000066000000}"/>
+    <cellStyle name="標準 2 62" xfId="103" xr:uid="{00000000-0005-0000-0000-000067000000}"/>
+    <cellStyle name="標準 2 63" xfId="104" xr:uid="{00000000-0005-0000-0000-000068000000}"/>
+    <cellStyle name="標準 2 64" xfId="105" xr:uid="{00000000-0005-0000-0000-000069000000}"/>
+    <cellStyle name="標準 2 65" xfId="106" xr:uid="{00000000-0005-0000-0000-00006A000000}"/>
+    <cellStyle name="標準 2 66" xfId="107" xr:uid="{00000000-0005-0000-0000-00006B000000}"/>
+    <cellStyle name="標準 2 67" xfId="108" xr:uid="{00000000-0005-0000-0000-00006C000000}"/>
+    <cellStyle name="標準 2 68" xfId="109" xr:uid="{00000000-0005-0000-0000-00006D000000}"/>
+    <cellStyle name="標準 2 69" xfId="110" xr:uid="{00000000-0005-0000-0000-00006E000000}"/>
+    <cellStyle name="標準 2 7" xfId="111" xr:uid="{00000000-0005-0000-0000-00006F000000}"/>
+    <cellStyle name="標準 2 70" xfId="112" xr:uid="{00000000-0005-0000-0000-000070000000}"/>
+    <cellStyle name="標準 2 71" xfId="113" xr:uid="{00000000-0005-0000-0000-000071000000}"/>
+    <cellStyle name="標準 2 72" xfId="114" xr:uid="{00000000-0005-0000-0000-000072000000}"/>
+    <cellStyle name="標準 2 73" xfId="115" xr:uid="{00000000-0005-0000-0000-000073000000}"/>
+    <cellStyle name="標準 2 74" xfId="116" xr:uid="{00000000-0005-0000-0000-000074000000}"/>
+    <cellStyle name="標準 2 75" xfId="117" xr:uid="{00000000-0005-0000-0000-000075000000}"/>
+    <cellStyle name="標準 2 76" xfId="118" xr:uid="{00000000-0005-0000-0000-000076000000}"/>
+    <cellStyle name="標準 2 77" xfId="119" xr:uid="{00000000-0005-0000-0000-000077000000}"/>
+    <cellStyle name="標準 2 78" xfId="120" xr:uid="{00000000-0005-0000-0000-000078000000}"/>
+    <cellStyle name="標準 2 79" xfId="121" xr:uid="{00000000-0005-0000-0000-000079000000}"/>
+    <cellStyle name="標準 2 8" xfId="122" xr:uid="{00000000-0005-0000-0000-00007A000000}"/>
+    <cellStyle name="標準 2 80" xfId="123" xr:uid="{00000000-0005-0000-0000-00007B000000}"/>
+    <cellStyle name="標準 2 81" xfId="124" xr:uid="{00000000-0005-0000-0000-00007C000000}"/>
+    <cellStyle name="標準 2 82" xfId="125" xr:uid="{00000000-0005-0000-0000-00007D000000}"/>
+    <cellStyle name="標準 2 83" xfId="126" xr:uid="{00000000-0005-0000-0000-00007E000000}"/>
+    <cellStyle name="標準 2 84" xfId="127" xr:uid="{00000000-0005-0000-0000-00007F000000}"/>
+    <cellStyle name="標準 2 85" xfId="128" xr:uid="{00000000-0005-0000-0000-000080000000}"/>
+    <cellStyle name="標準 2 86" xfId="129" xr:uid="{00000000-0005-0000-0000-000081000000}"/>
+    <cellStyle name="標準 2 87" xfId="130" xr:uid="{00000000-0005-0000-0000-000082000000}"/>
+    <cellStyle name="標準 2 88" xfId="131" xr:uid="{00000000-0005-0000-0000-000083000000}"/>
+    <cellStyle name="標準 2 89" xfId="132" xr:uid="{00000000-0005-0000-0000-000084000000}"/>
+    <cellStyle name="標準 2 9" xfId="133" xr:uid="{00000000-0005-0000-0000-000085000000}"/>
+    <cellStyle name="標準 2 90" xfId="134" xr:uid="{00000000-0005-0000-0000-000086000000}"/>
+    <cellStyle name="標準 2 91" xfId="135" xr:uid="{00000000-0005-0000-0000-000087000000}"/>
+    <cellStyle name="標準 2 92" xfId="136" xr:uid="{00000000-0005-0000-0000-000088000000}"/>
+    <cellStyle name="標準 2 93" xfId="137" xr:uid="{00000000-0005-0000-0000-000089000000}"/>
+    <cellStyle name="標準 2 94" xfId="138" xr:uid="{00000000-0005-0000-0000-00008A000000}"/>
+    <cellStyle name="標準 2 95" xfId="139" xr:uid="{00000000-0005-0000-0000-00008B000000}"/>
+    <cellStyle name="標準 2 96" xfId="140" xr:uid="{00000000-0005-0000-0000-00008C000000}"/>
+    <cellStyle name="標準 2 97" xfId="141" xr:uid="{00000000-0005-0000-0000-00008D000000}"/>
+    <cellStyle name="標準 2 98" xfId="142" xr:uid="{00000000-0005-0000-0000-00008E000000}"/>
+    <cellStyle name="標準 2 99" xfId="143" xr:uid="{00000000-0005-0000-0000-00008F000000}"/>
+    <cellStyle name="標準 3" xfId="144" xr:uid="{00000000-0005-0000-0000-000090000000}"/>
+    <cellStyle name="標準 4" xfId="145" xr:uid="{00000000-0005-0000-0000-000091000000}"/>
+    <cellStyle name="標準 5" xfId="146" xr:uid="{00000000-0005-0000-0000-000092000000}"/>
+    <cellStyle name="標準 6" xfId="147" xr:uid="{00000000-0005-0000-0000-000093000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1255,7 +1254,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1330,6 +1329,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -1365,6 +1381,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1540,1377 +1573,1377 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E82"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" style="9" customWidth="1"/>
-    <col min="2" max="2" width="45.88671875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="6.77734375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.21875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="45.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="3"/>
+    <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.15">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:5" ht="15">
+      <c r="A1" s="24" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" s="25" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="28" t="s">
+    <row r="3" spans="1:5" ht="17.25" customHeight="1">
+      <c r="A3" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="E3" s="6"/>
-    </row>
-    <row r="4" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="29"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="7" t="s">
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:5" ht="17.25" customHeight="1">
+      <c r="A4" s="27"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A5" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="9">
         <v>582</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="10">
         <v>3190396706</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="11">
         <v>273085707</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A6" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="9">
         <v>522</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="10">
         <v>3064100061</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="11">
         <v>262563958</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A7" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="9">
         <v>581</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="10">
         <v>2686407772</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="11">
         <v>218455127</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A8" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="9">
         <v>521</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="10">
         <v>2560111127</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="11">
         <v>207933378</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A9" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="9">
         <v>517</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="10">
         <v>2836921138</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="11">
         <v>249729003</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A10" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="9">
         <v>350</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="10">
         <v>2163299424</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="11">
         <v>194185426</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A11" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="9">
         <v>236</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="10">
         <v>837777792</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="11">
         <v>69058233</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A12" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="9">
         <v>60</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="10">
         <v>126296645</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="11">
         <v>10521749</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A13" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="9">
         <v>176</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="10">
         <v>711481147</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="11">
         <v>58536484</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A14" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="9">
         <v>13</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="10">
         <v>68149976</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="11">
         <v>4972929</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A15" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="9">
         <v>29</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="10">
         <v>63474625</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="11">
         <v>4781651</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A16" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="9">
         <v>15</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="10">
         <v>35700683</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="11">
         <v>2790765</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A17" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="9">
         <v>9</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="10">
         <v>79333024</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="11">
         <v>6042430</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="9">
         <v>7</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="10">
         <v>40174994</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="11">
         <v>3192467</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A19" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="9">
         <v>44</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="10">
         <v>90779258</v>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="11">
         <v>7657691</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A20" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="9">
         <v>29</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="10">
         <v>60100312</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="11">
         <v>5286246</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A21" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="9">
         <v>17</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="10">
         <v>33431502</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="11">
         <v>2732271</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A22" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="9">
         <v>16</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="10">
         <v>30495650</v>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="11">
         <v>2444738</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10" t="s">
+    <row r="23" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A23" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="9">
         <v>20</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="10">
         <v>38497685</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="11">
         <v>2880971</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A24" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="9">
         <v>17</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="10">
         <v>75224349</v>
       </c>
-      <c r="E24" s="13">
+      <c r="E24" s="11">
         <v>5817690</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A25" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="9">
         <v>29</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="10">
         <v>112214782</v>
       </c>
-      <c r="E25" s="13">
+      <c r="E25" s="11">
         <v>9435771</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A26" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="9">
         <v>17</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="10">
         <v>52027047</v>
       </c>
-      <c r="E26" s="13">
+      <c r="E26" s="11">
         <v>3967697</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A27" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="9">
         <v>9</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="10">
         <v>37859433</v>
       </c>
-      <c r="E27" s="13">
+      <c r="E27" s="11">
         <v>2992907</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A28" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="9">
         <v>25</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="10">
         <v>146611117</v>
       </c>
-      <c r="E28" s="13">
+      <c r="E28" s="11">
         <v>14583758</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="10" t="s">
+    <row r="29" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A29" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="9">
         <v>21</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="10">
         <v>685773216</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E29" s="11">
         <v>75366780</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A30" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="9">
         <v>20</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="10">
         <v>181784282</v>
       </c>
-      <c r="E30" s="13">
+      <c r="E30" s="11">
         <v>20736200</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A31" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="9">
         <v>4</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="10">
         <v>584936605</v>
       </c>
-      <c r="E31" s="13">
+      <c r="E31" s="11">
         <v>67010021</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A32" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B32" s="23" t="s">
+      <c r="B32" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="9">
         <v>3</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="10">
         <v>80947671</v>
       </c>
-      <c r="E32" s="13">
+      <c r="E32" s="11">
         <v>12379441</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="10" t="s">
+    <row r="33" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A33" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="9">
         <v>17</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="10">
         <v>100836611</v>
       </c>
-      <c r="E33" s="13">
+      <c r="E33" s="11">
         <v>8356759</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A34" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="9">
         <v>6</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="10">
         <v>221145728</v>
       </c>
-      <c r="E34" s="13">
+      <c r="E34" s="11">
         <v>15159635</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A35" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="B35" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="9">
         <v>1</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="10">
         <v>108710567</v>
       </c>
-      <c r="E35" s="13">
+      <c r="E35" s="11">
         <v>7148165</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A36" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="B36" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="9">
         <v>2</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="10">
         <v>48173221</v>
       </c>
-      <c r="E36" s="13">
+      <c r="E36" s="11">
         <v>4135406</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A37" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="9">
         <v>1</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="10">
         <v>12158452</v>
       </c>
-      <c r="E37" s="13">
+      <c r="E37" s="11">
         <v>168433</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="10" t="s">
+    <row r="38" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A38" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C38" s="11">
+      <c r="C38" s="9">
         <v>2</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="10">
         <v>52103488</v>
       </c>
-      <c r="E38" s="13">
+      <c r="E38" s="11">
         <v>3707631</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="10" t="s">
+    <row r="39" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A39" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="9">
         <v>48</v>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="10">
         <v>123411836</v>
       </c>
-      <c r="E39" s="13">
+      <c r="E39" s="11">
         <v>9161484</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="10" t="s">
+    <row r="40" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A40" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C40" s="11">
+      <c r="C40" s="9">
         <v>13</v>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="10">
         <v>42179255</v>
       </c>
-      <c r="E40" s="13">
+      <c r="E40" s="11">
         <v>3018244</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="10" t="s">
+    <row r="41" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A41" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="9">
         <v>4</v>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="10">
         <v>6577565</v>
       </c>
-      <c r="E41" s="13">
+      <c r="E41" s="11">
         <v>506006</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="10" t="s">
+    <row r="42" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A42" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C42" s="11">
+      <c r="C42" s="9">
         <v>5</v>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="10">
         <v>8613708</v>
       </c>
-      <c r="E42" s="13">
+      <c r="E42" s="11">
         <v>638379</v>
       </c>
     </row>
-    <row r="43" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="10" t="s">
+    <row r="43" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A43" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B43" s="22" t="s">
+      <c r="B43" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="9">
         <v>11</v>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="10">
         <v>23738356</v>
       </c>
-      <c r="E43" s="13">
+      <c r="E43" s="11">
         <v>2004097</v>
       </c>
     </row>
-    <row r="44" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="10" t="s">
+    <row r="44" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A44" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="9">
         <v>11</v>
       </c>
-      <c r="D44" s="12">
+      <c r="D44" s="10">
         <v>33518214</v>
       </c>
-      <c r="E44" s="13">
+      <c r="E44" s="11">
         <v>2367766</v>
       </c>
     </row>
-    <row r="45" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="15" t="s">
+    <row r="45" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A45" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B45" s="24" t="s">
+      <c r="B45" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C45" s="16">
+      <c r="C45" s="14">
         <v>4</v>
       </c>
-      <c r="D45" s="17">
+      <c r="D45" s="15">
         <v>8784738</v>
       </c>
-      <c r="E45" s="18">
+      <c r="E45" s="16">
         <v>626992</v>
       </c>
     </row>
-    <row r="46" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="19" t="s">
+    <row r="46" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A46" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="B46" s="20" t="s">
+      <c r="B46" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C46" s="11">
+      <c r="C46" s="9">
         <v>64</v>
       </c>
-      <c r="D46" s="12">
+      <c r="D46" s="10">
         <v>112584877</v>
       </c>
-      <c r="E46" s="13">
+      <c r="E46" s="11">
         <v>10242306</v>
       </c>
     </row>
-    <row r="47" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="10" t="s">
+    <row r="47" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A47" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B47" s="22" t="s">
+      <c r="B47" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="9">
         <v>28</v>
       </c>
-      <c r="D47" s="12">
+      <c r="D47" s="10">
         <v>48397154</v>
       </c>
-      <c r="E47" s="13">
+      <c r="E47" s="11">
         <v>4653890</v>
       </c>
     </row>
-    <row r="48" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="10" t="s">
+    <row r="48" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A48" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B48" s="23" t="s">
+      <c r="B48" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C48" s="11">
+      <c r="C48" s="9">
         <v>2</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="10">
         <v>1341826</v>
       </c>
-      <c r="E48" s="13">
+      <c r="E48" s="11">
         <v>140588</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="10" t="s">
+    <row r="49" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A49" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B49" s="23" t="s">
+      <c r="B49" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="9">
         <v>26</v>
       </c>
-      <c r="D49" s="12">
+      <c r="D49" s="10">
         <v>47055328</v>
       </c>
-      <c r="E49" s="13">
+      <c r="E49" s="11">
         <v>4513302</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="10" t="s">
+    <row r="50" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A50" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B50" s="22" t="s">
+      <c r="B50" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C50" s="11">
+      <c r="C50" s="9">
         <v>19</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="10">
         <v>33461117</v>
       </c>
-      <c r="E50" s="13">
+      <c r="E50" s="11">
         <v>2825186</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="10" t="s">
+    <row r="51" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A51" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B51" s="23" t="s">
+      <c r="B51" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="9">
         <v>12</v>
       </c>
-      <c r="D51" s="12">
+      <c r="D51" s="10">
         <v>22528451</v>
       </c>
-      <c r="E51" s="13">
+      <c r="E51" s="11">
         <v>1987378</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="10" t="s">
+    <row r="52" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A52" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B52" s="23" t="s">
+      <c r="B52" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C52" s="11">
+      <c r="C52" s="9">
         <v>7</v>
       </c>
-      <c r="D52" s="12">
+      <c r="D52" s="10">
         <v>10932666</v>
       </c>
-      <c r="E52" s="13">
+      <c r="E52" s="11">
         <v>837808</v>
       </c>
     </row>
-    <row r="53" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="10" t="s">
+    <row r="53" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A53" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B53" s="22" t="s">
+      <c r="B53" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C53" s="11">
+      <c r="C53" s="9">
         <v>6</v>
       </c>
-      <c r="D53" s="12">
+      <c r="D53" s="10">
         <v>15357481</v>
       </c>
-      <c r="E53" s="13">
+      <c r="E53" s="11">
         <v>1279086</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="10" t="s">
+    <row r="54" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A54" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="B54" s="22" t="s">
+      <c r="B54" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C54" s="11">
+      <c r="C54" s="9">
         <v>7</v>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="10">
         <v>9128106</v>
       </c>
-      <c r="E54" s="13">
+      <c r="E54" s="11">
         <v>755444</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="10" t="s">
+    <row r="55" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A55" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B55" s="22" t="s">
+      <c r="B55" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="9">
         <v>4</v>
       </c>
-      <c r="D55" s="12">
+      <c r="D55" s="10">
         <v>6241019</v>
       </c>
-      <c r="E55" s="13">
+      <c r="E55" s="11">
         <v>728700</v>
       </c>
     </row>
-    <row r="56" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="10" t="s">
+    <row r="56" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A56" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B56" s="20" t="s">
+      <c r="B56" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C56" s="11">
+      <c r="C56" s="9">
         <v>29</v>
       </c>
-      <c r="D56" s="12">
+      <c r="D56" s="10">
         <v>152330482</v>
       </c>
-      <c r="E56" s="13">
+      <c r="E56" s="11">
         <v>12860804</v>
       </c>
     </row>
-    <row r="57" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="10" t="s">
+    <row r="57" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A57" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B57" s="22" t="s">
+      <c r="B57" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="9">
         <v>13</v>
       </c>
-      <c r="D57" s="12">
+      <c r="D57" s="10">
         <v>40726717</v>
       </c>
-      <c r="E57" s="13">
+      <c r="E57" s="11">
         <v>3193035</v>
       </c>
     </row>
-    <row r="58" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="10" t="s">
+    <row r="58" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A58" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B58" s="22" t="s">
+      <c r="B58" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="11">
+      <c r="C58" s="9">
         <v>12</v>
       </c>
-      <c r="D58" s="12">
+      <c r="D58" s="10">
         <v>28947320</v>
       </c>
-      <c r="E58" s="13">
+      <c r="E58" s="11">
         <v>2209442</v>
       </c>
     </row>
-    <row r="59" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="10" t="s">
+    <row r="59" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A59" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B59" s="22" t="s">
+      <c r="B59" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="11">
+      <c r="C59" s="9">
         <v>4</v>
       </c>
-      <c r="D59" s="12">
+      <c r="D59" s="10">
         <v>82656445</v>
       </c>
-      <c r="E59" s="13">
+      <c r="E59" s="11">
         <v>7458327</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="10" t="s">
+    <row r="60" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A60" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="B60" s="20" t="s">
+      <c r="B60" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="11">
+      <c r="C60" s="9">
         <v>42</v>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="10">
         <v>476190801</v>
       </c>
-      <c r="E60" s="13">
+      <c r="E60" s="11">
         <v>27504214</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="10" t="s">
+    <row r="61" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A61" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="B61" s="22" t="s">
+      <c r="B61" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="C61" s="11">
+      <c r="C61" s="9">
         <v>14</v>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="10">
         <v>53231261</v>
       </c>
-      <c r="E61" s="13">
+      <c r="E61" s="11">
         <v>6407393</v>
       </c>
     </row>
-    <row r="62" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="10" t="s">
+    <row r="62" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A62" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B62" s="22" t="s">
+      <c r="B62" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="C62" s="11">
+      <c r="C62" s="9">
         <v>22</v>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="10">
         <v>282263274</v>
       </c>
-      <c r="E62" s="13">
+      <c r="E62" s="11">
         <v>11678188</v>
       </c>
     </row>
-    <row r="63" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="10" t="s">
+    <row r="63" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A63" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B63" s="22" t="s">
+      <c r="B63" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C63" s="11">
+      <c r="C63" s="9">
         <v>6</v>
       </c>
-      <c r="D63" s="12">
+      <c r="D63" s="10">
         <v>140696266</v>
       </c>
-      <c r="E63" s="13">
+      <c r="E63" s="11">
         <v>9418633</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="10" t="s">
+    <row r="64" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A64" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B64" s="20" t="s">
+      <c r="B64" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C64" s="11">
+      <c r="C64" s="9">
         <v>14</v>
       </c>
-      <c r="D64" s="12">
+      <c r="D64" s="10">
         <v>97001854</v>
       </c>
-      <c r="E64" s="13">
+      <c r="E64" s="11">
         <v>12688115</v>
       </c>
     </row>
-    <row r="65" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="10" t="s">
+    <row r="65" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A65" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B65" s="22" t="s">
+      <c r="B65" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C65" s="11">
+      <c r="C65" s="9">
         <v>9</v>
       </c>
-      <c r="D65" s="12">
+      <c r="D65" s="10">
         <v>68010600</v>
       </c>
-      <c r="E65" s="13">
+      <c r="E65" s="11">
         <v>8826147</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="10" t="s">
+    <row r="66" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A66" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B66" s="22" t="s">
+      <c r="B66" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C66" s="11">
+      <c r="C66" s="9">
         <v>2</v>
       </c>
-      <c r="D66" s="12">
+      <c r="D66" s="10">
         <v>2197039</v>
       </c>
-      <c r="E66" s="13">
+      <c r="E66" s="11">
         <v>157861</v>
       </c>
     </row>
-    <row r="67" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="10" t="s">
+    <row r="67" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A67" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B67" s="22" t="s">
+      <c r="B67" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C67" s="11">
+      <c r="C67" s="9">
         <v>3</v>
       </c>
-      <c r="D67" s="12">
+      <c r="D67" s="10">
         <v>26794215</v>
       </c>
-      <c r="E67" s="13">
+      <c r="E67" s="11">
         <v>3704107</v>
       </c>
     </row>
-    <row r="68" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="10" t="s">
+    <row r="68" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A68" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B68" s="20" t="s">
+      <c r="B68" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C68" s="11">
+      <c r="C68" s="9">
         <v>74</v>
       </c>
-      <c r="D68" s="12">
+      <c r="D68" s="10">
         <v>290669386</v>
       </c>
-      <c r="E68" s="13">
+      <c r="E68" s="11">
         <v>25648217</v>
       </c>
     </row>
-    <row r="69" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="10" t="s">
+    <row r="69" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A69" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B69" s="22" t="s">
+      <c r="B69" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C69" s="11">
+      <c r="C69" s="9">
         <v>9</v>
       </c>
-      <c r="D69" s="12">
+      <c r="D69" s="10">
         <v>24536787</v>
       </c>
-      <c r="E69" s="13">
+      <c r="E69" s="11">
         <v>2192670</v>
       </c>
     </row>
-    <row r="70" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="10" t="s">
+    <row r="70" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A70" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="B70" s="22" t="s">
+      <c r="B70" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C70" s="11">
+      <c r="C70" s="9">
         <v>29</v>
       </c>
-      <c r="D70" s="12">
+      <c r="D70" s="10">
         <v>65733216</v>
       </c>
-      <c r="E70" s="13">
+      <c r="E70" s="11">
         <v>4794238</v>
       </c>
     </row>
-    <row r="71" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="10" t="s">
+    <row r="71" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A71" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B71" s="22" t="s">
+      <c r="B71" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C71" s="11">
+      <c r="C71" s="9">
         <v>6</v>
       </c>
-      <c r="D71" s="12">
+      <c r="D71" s="10">
         <v>35138875</v>
       </c>
-      <c r="E71" s="13">
+      <c r="E71" s="11">
         <v>2856943</v>
       </c>
     </row>
-    <row r="72" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="10" t="s">
+    <row r="72" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A72" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B72" s="22" t="s">
+      <c r="B72" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="C72" s="11">
+      <c r="C72" s="9">
         <v>30</v>
       </c>
-      <c r="D72" s="12">
+      <c r="D72" s="10">
         <v>165260508</v>
       </c>
-      <c r="E72" s="13">
+      <c r="E72" s="11">
         <v>15804366</v>
       </c>
     </row>
-    <row r="73" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="10" t="s">
+    <row r="73" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A73" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="B73" s="20" t="s">
+      <c r="B73" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C73" s="11">
+      <c r="C73" s="9">
         <v>48</v>
       </c>
-      <c r="D73" s="12">
+      <c r="D73" s="10">
         <v>193510734</v>
       </c>
-      <c r="E73" s="13">
+      <c r="E73" s="11">
         <v>15395919</v>
       </c>
     </row>
-    <row r="74" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="10" t="s">
+    <row r="74" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A74" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="B74" s="22" t="s">
+      <c r="B74" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C74" s="11">
+      <c r="C74" s="9">
         <v>6</v>
       </c>
-      <c r="D74" s="12">
+      <c r="D74" s="10">
         <v>35161552</v>
       </c>
-      <c r="E74" s="13">
+      <c r="E74" s="11">
         <v>3091569</v>
       </c>
     </row>
-    <row r="75" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="10" t="s">
+    <row r="75" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A75" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B75" s="22" t="s">
+      <c r="B75" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C75" s="11">
+      <c r="C75" s="9">
         <v>23</v>
       </c>
-      <c r="D75" s="12">
+      <c r="D75" s="10">
         <v>51225533</v>
       </c>
-      <c r="E75" s="13">
+      <c r="E75" s="11">
         <v>4222145</v>
       </c>
     </row>
-    <row r="76" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="10" t="s">
+    <row r="76" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A76" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B76" s="22" t="s">
+      <c r="B76" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C76" s="11">
+      <c r="C76" s="9">
         <v>8</v>
       </c>
-      <c r="D76" s="12">
+      <c r="D76" s="10">
         <v>20181956</v>
       </c>
-      <c r="E76" s="13">
+      <c r="E76" s="11">
         <v>2039792</v>
       </c>
     </row>
-    <row r="77" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="10" t="s">
+    <row r="77" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A77" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="B77" s="22" t="s">
+      <c r="B77" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C77" s="11">
+      <c r="C77" s="9">
         <v>2</v>
       </c>
-      <c r="D77" s="12">
+      <c r="D77" s="10">
         <v>12596598</v>
       </c>
-      <c r="E77" s="13">
+      <c r="E77" s="11">
         <v>771262</v>
       </c>
     </row>
-    <row r="78" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="10" t="s">
+    <row r="78" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A78" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B78" s="22" t="s">
+      <c r="B78" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C78" s="11">
+      <c r="C78" s="9">
         <v>9</v>
       </c>
-      <c r="D78" s="12">
+      <c r="D78" s="10">
         <v>74345095</v>
       </c>
-      <c r="E78" s="13">
+      <c r="E78" s="11">
         <v>5271151</v>
       </c>
     </row>
-    <row r="79" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="10" t="s">
+    <row r="79" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A79" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="B79" s="25" t="s">
+      <c r="B79" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="C79" s="11">
+      <c r="C79" s="9">
         <v>5</v>
       </c>
-      <c r="D79" s="12">
+      <c r="D79" s="10">
         <v>227178923</v>
       </c>
-      <c r="E79" s="13">
+      <c r="E79" s="11">
         <v>12834955</v>
       </c>
     </row>
-    <row r="80" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="10" t="s">
+    <row r="80" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A80" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="B80" s="25" t="s">
+      <c r="B80" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="C80" s="11">
+      <c r="C80" s="9">
         <v>25</v>
       </c>
-      <c r="D80" s="12">
+      <c r="D80" s="10">
         <v>120648071</v>
       </c>
-      <c r="E80" s="13">
+      <c r="E80" s="11">
         <v>14375183</v>
       </c>
     </row>
-    <row r="81" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="10" t="s">
+    <row r="81" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A81" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="B81" s="25" t="s">
+      <c r="B81" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="C81" s="11">
+      <c r="C81" s="9">
         <v>77</v>
       </c>
-      <c r="D81" s="12">
+      <c r="D81" s="10">
         <v>308848382</v>
       </c>
-      <c r="E81" s="13">
+      <c r="E81" s="11">
         <v>28214286</v>
       </c>
     </row>
-    <row r="82" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="15" t="s">
+    <row r="82" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A82" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="B82" s="4" t="s">
+      <c r="B82" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="C82" s="16">
+      <c r="C82" s="14">
         <v>7</v>
       </c>
-      <c r="D82" s="17">
+      <c r="D82" s="15">
         <v>159473833</v>
       </c>
-      <c r="E82" s="18">
+      <c r="E82" s="16">
         <v>10773016</v>
       </c>
     </row>
@@ -2937,1377 +2970,1377 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E82"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" style="9" customWidth="1"/>
-    <col min="2" max="2" width="45.88671875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="6.77734375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.21875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="45.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="3"/>
+    <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.15">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:5" ht="15">
+      <c r="A1" s="24" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" s="25" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="28" t="s">
+    <row r="3" spans="1:5" ht="17.25" customHeight="1">
+      <c r="A3" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="E3" s="6"/>
-    </row>
-    <row r="4" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="29"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="7" t="s">
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:5" ht="17.25" customHeight="1">
+      <c r="A4" s="27"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A5" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="9">
         <v>582</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="10">
         <v>10000</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="11">
         <v>10000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A6" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="9">
         <v>522</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="10">
         <v>9604</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="11">
         <v>9615</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A7" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="9">
         <v>581</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="10">
         <v>8420</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="11">
         <v>8000</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A8" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="9">
         <v>521</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="10">
         <v>8024</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="11">
         <v>7614</v>
       </c>
     </row>
-    <row r="9" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A9" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="9">
         <v>517</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="10">
         <v>8892</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="11">
         <v>9145</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A10" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="9">
         <v>350</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="10">
         <v>6781</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="11">
         <v>7111</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A11" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="9">
         <v>236</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="10">
         <v>2626</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="11">
         <v>2529</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A12" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="9">
         <v>60</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="10">
         <v>396</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="11">
         <v>385</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A13" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="9">
         <v>176</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="10">
         <v>2230</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="11">
         <v>2144</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A14" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="9">
         <v>13</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="10">
         <v>214</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="11">
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A15" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="9">
         <v>29</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="10">
         <v>199</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="11">
         <v>175</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A16" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="9">
         <v>15</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="10">
         <v>112</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="11">
         <v>102</v>
       </c>
     </row>
-    <row r="17" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="10" t="s">
+    <row r="17" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A17" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="9">
         <v>9</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="10">
         <v>249</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="11">
         <v>221</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A18" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="9">
         <v>7</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="10">
         <v>126</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="11">
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="10" t="s">
+    <row r="19" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A19" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="9">
         <v>44</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="10">
         <v>285</v>
       </c>
-      <c r="E19" s="13">
+      <c r="E19" s="11">
         <v>280</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A20" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="9">
         <v>29</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="10">
         <v>188</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="11">
         <v>194</v>
       </c>
     </row>
-    <row r="21" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10" t="s">
+    <row r="21" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A21" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="9">
         <v>17</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="10">
         <v>105</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="11">
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A22" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="9">
         <v>16</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="10">
         <v>96</v>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="11">
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10" t="s">
+    <row r="23" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A23" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="9">
         <v>20</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="10">
         <v>121</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="11">
         <v>105</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A24" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="9">
         <v>17</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="10">
         <v>236</v>
       </c>
-      <c r="E24" s="13">
+      <c r="E24" s="11">
         <v>213</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
+    <row r="25" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A25" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="9">
         <v>29</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="10">
         <v>352</v>
       </c>
-      <c r="E25" s="13">
+      <c r="E25" s="11">
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A26" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="9">
         <v>17</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="10">
         <v>163</v>
       </c>
-      <c r="E26" s="13">
+      <c r="E26" s="11">
         <v>145</v>
       </c>
     </row>
-    <row r="27" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A27" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="9">
         <v>9</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="10">
         <v>119</v>
       </c>
-      <c r="E27" s="13">
+      <c r="E27" s="11">
         <v>110</v>
       </c>
     </row>
-    <row r="28" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A28" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="9">
         <v>25</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="10">
         <v>460</v>
       </c>
-      <c r="E28" s="13">
+      <c r="E28" s="11">
         <v>534</v>
       </c>
     </row>
-    <row r="29" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="10" t="s">
+    <row r="29" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A29" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="9">
         <v>21</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="10">
         <v>2149</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E29" s="11">
         <v>2760</v>
       </c>
     </row>
-    <row r="30" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A30" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="9">
         <v>20</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="10">
         <v>570</v>
       </c>
-      <c r="E30" s="13">
+      <c r="E30" s="11">
         <v>759</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A31" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="9">
         <v>4</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="10">
         <v>1833</v>
       </c>
-      <c r="E31" s="13">
+      <c r="E31" s="11">
         <v>2454</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A32" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B32" s="23" t="s">
+      <c r="B32" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="9">
         <v>3</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="10">
         <v>254</v>
       </c>
-      <c r="E32" s="13">
+      <c r="E32" s="11">
         <v>453</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="10" t="s">
+    <row r="33" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A33" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="9">
         <v>17</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="10">
         <v>316</v>
       </c>
-      <c r="E33" s="13">
+      <c r="E33" s="11">
         <v>306</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A34" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="9">
         <v>6</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="10">
         <v>693</v>
       </c>
-      <c r="E34" s="13">
+      <c r="E34" s="11">
         <v>555</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A35" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="B35" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="9">
         <v>1</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="10">
         <v>341</v>
       </c>
-      <c r="E35" s="13">
+      <c r="E35" s="11">
         <v>262</v>
       </c>
     </row>
-    <row r="36" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A36" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="B36" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="9">
         <v>2</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="10">
         <v>151</v>
       </c>
-      <c r="E36" s="13">
+      <c r="E36" s="11">
         <v>151</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A37" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="9">
         <v>1</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="10">
         <v>38</v>
       </c>
-      <c r="E37" s="13">
+      <c r="E37" s="11">
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="10" t="s">
+    <row r="38" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A38" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C38" s="11">
+      <c r="C38" s="9">
         <v>2</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="10">
         <v>163</v>
       </c>
-      <c r="E38" s="13">
+      <c r="E38" s="11">
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="10" t="s">
+    <row r="39" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A39" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C39" s="11">
+      <c r="C39" s="9">
         <v>48</v>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="10">
         <v>387</v>
       </c>
-      <c r="E39" s="13">
+      <c r="E39" s="11">
         <v>335</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="10" t="s">
+    <row r="40" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A40" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C40" s="11">
+      <c r="C40" s="9">
         <v>13</v>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="10">
         <v>132</v>
       </c>
-      <c r="E40" s="13">
+      <c r="E40" s="11">
         <v>111</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="10" t="s">
+    <row r="41" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A41" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="9">
         <v>4</v>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="10">
         <v>21</v>
       </c>
-      <c r="E41" s="13">
+      <c r="E41" s="11">
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="10" t="s">
+    <row r="42" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A42" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C42" s="11">
+      <c r="C42" s="9">
         <v>5</v>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="10">
         <v>27</v>
       </c>
-      <c r="E42" s="13">
+      <c r="E42" s="11">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="10" t="s">
+    <row r="43" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A43" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B43" s="22" t="s">
+      <c r="B43" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C43" s="11">
+      <c r="C43" s="9">
         <v>11</v>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="10">
         <v>74</v>
       </c>
-      <c r="E43" s="13">
+      <c r="E43" s="11">
         <v>73</v>
       </c>
     </row>
-    <row r="44" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="10" t="s">
+    <row r="44" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A44" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="C44" s="11">
+      <c r="C44" s="9">
         <v>11</v>
       </c>
-      <c r="D44" s="12">
+      <c r="D44" s="10">
         <v>105</v>
       </c>
-      <c r="E44" s="13">
+      <c r="E44" s="11">
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="15" t="s">
+    <row r="45" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A45" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B45" s="24" t="s">
+      <c r="B45" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C45" s="16">
+      <c r="C45" s="14">
         <v>4</v>
       </c>
-      <c r="D45" s="17">
+      <c r="D45" s="15">
         <v>28</v>
       </c>
-      <c r="E45" s="18">
+      <c r="E45" s="16">
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="19" t="s">
+    <row r="46" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A46" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="B46" s="20" t="s">
+      <c r="B46" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C46" s="11">
+      <c r="C46" s="9">
         <v>64</v>
       </c>
-      <c r="D46" s="12">
+      <c r="D46" s="10">
         <v>353</v>
       </c>
-      <c r="E46" s="13">
+      <c r="E46" s="11">
         <v>375</v>
       </c>
     </row>
-    <row r="47" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="10" t="s">
+    <row r="47" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A47" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B47" s="22" t="s">
+      <c r="B47" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C47" s="11">
+      <c r="C47" s="9">
         <v>28</v>
       </c>
-      <c r="D47" s="12">
+      <c r="D47" s="10">
         <v>152</v>
       </c>
-      <c r="E47" s="13">
+      <c r="E47" s="11">
         <v>170</v>
       </c>
     </row>
-    <row r="48" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="10" t="s">
+    <row r="48" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A48" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B48" s="23" t="s">
+      <c r="B48" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C48" s="11">
+      <c r="C48" s="9">
         <v>2</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="10">
         <v>4</v>
       </c>
-      <c r="E48" s="13">
+      <c r="E48" s="11">
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="10" t="s">
+    <row r="49" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A49" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B49" s="23" t="s">
+      <c r="B49" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="C49" s="11">
+      <c r="C49" s="9">
         <v>26</v>
       </c>
-      <c r="D49" s="12">
+      <c r="D49" s="10">
         <v>147</v>
       </c>
-      <c r="E49" s="13">
+      <c r="E49" s="11">
         <v>165</v>
       </c>
     </row>
-    <row r="50" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="10" t="s">
+    <row r="50" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A50" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B50" s="22" t="s">
+      <c r="B50" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="C50" s="11">
+      <c r="C50" s="9">
         <v>19</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="10">
         <v>105</v>
       </c>
-      <c r="E50" s="13">
+      <c r="E50" s="11">
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="10" t="s">
+    <row r="51" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A51" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B51" s="23" t="s">
+      <c r="B51" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C51" s="11">
+      <c r="C51" s="9">
         <v>12</v>
       </c>
-      <c r="D51" s="12">
+      <c r="D51" s="10">
         <v>71</v>
       </c>
-      <c r="E51" s="13">
+      <c r="E51" s="11">
         <v>73</v>
       </c>
     </row>
-    <row r="52" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="10" t="s">
+    <row r="52" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A52" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B52" s="23" t="s">
+      <c r="B52" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C52" s="11">
+      <c r="C52" s="9">
         <v>7</v>
       </c>
-      <c r="D52" s="12">
+      <c r="D52" s="10">
         <v>34</v>
       </c>
-      <c r="E52" s="13">
+      <c r="E52" s="11">
         <v>31</v>
       </c>
     </row>
-    <row r="53" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="10" t="s">
+    <row r="53" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A53" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B53" s="22" t="s">
+      <c r="B53" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C53" s="11">
+      <c r="C53" s="9">
         <v>6</v>
       </c>
-      <c r="D53" s="12">
+      <c r="D53" s="10">
         <v>48</v>
       </c>
-      <c r="E53" s="13">
+      <c r="E53" s="11">
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="10" t="s">
+    <row r="54" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A54" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="B54" s="22" t="s">
+      <c r="B54" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C54" s="11">
+      <c r="C54" s="9">
         <v>7</v>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="10">
         <v>29</v>
       </c>
-      <c r="E54" s="13">
+      <c r="E54" s="11">
         <v>28</v>
       </c>
     </row>
-    <row r="55" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="10" t="s">
+    <row r="55" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A55" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B55" s="22" t="s">
+      <c r="B55" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="9">
         <v>4</v>
       </c>
-      <c r="D55" s="12">
+      <c r="D55" s="10">
         <v>20</v>
       </c>
-      <c r="E55" s="13">
+      <c r="E55" s="11">
         <v>27</v>
       </c>
     </row>
-    <row r="56" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="10" t="s">
+    <row r="56" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A56" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B56" s="20" t="s">
+      <c r="B56" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="C56" s="11">
+      <c r="C56" s="9">
         <v>29</v>
       </c>
-      <c r="D56" s="12">
+      <c r="D56" s="10">
         <v>477</v>
       </c>
-      <c r="E56" s="13">
+      <c r="E56" s="11">
         <v>471</v>
       </c>
     </row>
-    <row r="57" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="10" t="s">
+    <row r="57" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A57" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B57" s="22" t="s">
+      <c r="B57" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="9">
         <v>13</v>
       </c>
-      <c r="D57" s="12">
+      <c r="D57" s="10">
         <v>128</v>
       </c>
-      <c r="E57" s="13">
+      <c r="E57" s="11">
         <v>117</v>
       </c>
     </row>
-    <row r="58" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="10" t="s">
+    <row r="58" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A58" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="B58" s="22" t="s">
+      <c r="B58" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="11">
+      <c r="C58" s="9">
         <v>12</v>
       </c>
-      <c r="D58" s="12">
+      <c r="D58" s="10">
         <v>91</v>
       </c>
-      <c r="E58" s="13">
+      <c r="E58" s="11">
         <v>81</v>
       </c>
     </row>
-    <row r="59" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="10" t="s">
+    <row r="59" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A59" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B59" s="22" t="s">
+      <c r="B59" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C59" s="11">
+      <c r="C59" s="9">
         <v>4</v>
       </c>
-      <c r="D59" s="12">
+      <c r="D59" s="10">
         <v>259</v>
       </c>
-      <c r="E59" s="13">
+      <c r="E59" s="11">
         <v>273</v>
       </c>
     </row>
-    <row r="60" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="10" t="s">
+    <row r="60" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A60" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="B60" s="20" t="s">
+      <c r="B60" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C60" s="11">
+      <c r="C60" s="9">
         <v>42</v>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="10">
         <v>1493</v>
       </c>
-      <c r="E60" s="13">
+      <c r="E60" s="11">
         <v>1007</v>
       </c>
     </row>
-    <row r="61" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="10" t="s">
+    <row r="61" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A61" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="B61" s="22" t="s">
+      <c r="B61" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="11">
+      <c r="C61" s="9">
         <v>14</v>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="10">
         <v>167</v>
       </c>
-      <c r="E61" s="13">
+      <c r="E61" s="11">
         <v>235</v>
       </c>
     </row>
-    <row r="62" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="10" t="s">
+    <row r="62" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A62" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B62" s="22" t="s">
+      <c r="B62" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="C62" s="11">
+      <c r="C62" s="9">
         <v>22</v>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="10">
         <v>885</v>
       </c>
-      <c r="E62" s="13">
+      <c r="E62" s="11">
         <v>428</v>
       </c>
     </row>
-    <row r="63" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="10" t="s">
+    <row r="63" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A63" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B63" s="22" t="s">
+      <c r="B63" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C63" s="11">
+      <c r="C63" s="9">
         <v>6</v>
       </c>
-      <c r="D63" s="12">
+      <c r="D63" s="10">
         <v>441</v>
       </c>
-      <c r="E63" s="13">
+      <c r="E63" s="11">
         <v>345</v>
       </c>
     </row>
-    <row r="64" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="10" t="s">
+    <row r="64" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A64" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B64" s="20" t="s">
+      <c r="B64" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C64" s="11">
+      <c r="C64" s="9">
         <v>14</v>
       </c>
-      <c r="D64" s="12">
+      <c r="D64" s="10">
         <v>304</v>
       </c>
-      <c r="E64" s="13">
+      <c r="E64" s="11">
         <v>465</v>
       </c>
     </row>
-    <row r="65" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="10" t="s">
+    <row r="65" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A65" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B65" s="22" t="s">
+      <c r="B65" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C65" s="11">
+      <c r="C65" s="9">
         <v>9</v>
       </c>
-      <c r="D65" s="12">
+      <c r="D65" s="10">
         <v>213</v>
       </c>
-      <c r="E65" s="13">
+      <c r="E65" s="11">
         <v>323</v>
       </c>
     </row>
-    <row r="66" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="10" t="s">
+    <row r="66" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A66" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B66" s="22" t="s">
+      <c r="B66" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C66" s="11">
+      <c r="C66" s="9">
         <v>2</v>
       </c>
-      <c r="D66" s="12">
+      <c r="D66" s="10">
         <v>7</v>
       </c>
-      <c r="E66" s="13">
+      <c r="E66" s="11">
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="10" t="s">
+    <row r="67" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A67" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B67" s="22" t="s">
+      <c r="B67" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C67" s="11">
+      <c r="C67" s="9">
         <v>3</v>
       </c>
-      <c r="D67" s="12">
+      <c r="D67" s="10">
         <v>84</v>
       </c>
-      <c r="E67" s="13">
+      <c r="E67" s="11">
         <v>136</v>
       </c>
     </row>
-    <row r="68" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="10" t="s">
+    <row r="68" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A68" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B68" s="20" t="s">
+      <c r="B68" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C68" s="11">
+      <c r="C68" s="9">
         <v>74</v>
       </c>
-      <c r="D68" s="12">
+      <c r="D68" s="10">
         <v>911</v>
       </c>
-      <c r="E68" s="13">
+      <c r="E68" s="11">
         <v>939</v>
       </c>
     </row>
-    <row r="69" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="10" t="s">
+    <row r="69" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A69" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B69" s="22" t="s">
+      <c r="B69" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C69" s="11">
+      <c r="C69" s="9">
         <v>9</v>
       </c>
-      <c r="D69" s="12">
+      <c r="D69" s="10">
         <v>77</v>
       </c>
-      <c r="E69" s="13">
+      <c r="E69" s="11">
         <v>80</v>
       </c>
     </row>
-    <row r="70" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="10" t="s">
+    <row r="70" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A70" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="B70" s="22" t="s">
+      <c r="B70" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C70" s="11">
+      <c r="C70" s="9">
         <v>29</v>
       </c>
-      <c r="D70" s="12">
+      <c r="D70" s="10">
         <v>206</v>
       </c>
-      <c r="E70" s="13">
+      <c r="E70" s="11">
         <v>176</v>
       </c>
     </row>
-    <row r="71" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="10" t="s">
+    <row r="71" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A71" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B71" s="22" t="s">
+      <c r="B71" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C71" s="11">
+      <c r="C71" s="9">
         <v>6</v>
       </c>
-      <c r="D71" s="12">
+      <c r="D71" s="10">
         <v>110</v>
       </c>
-      <c r="E71" s="13">
+      <c r="E71" s="11">
         <v>105</v>
       </c>
     </row>
-    <row r="72" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="10" t="s">
+    <row r="72" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A72" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B72" s="22" t="s">
+      <c r="B72" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="C72" s="11">
+      <c r="C72" s="9">
         <v>30</v>
       </c>
-      <c r="D72" s="12">
+      <c r="D72" s="10">
         <v>518</v>
       </c>
-      <c r="E72" s="13">
+      <c r="E72" s="11">
         <v>579</v>
       </c>
     </row>
-    <row r="73" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="10" t="s">
+    <row r="73" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A73" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="B73" s="20" t="s">
+      <c r="B73" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C73" s="11">
+      <c r="C73" s="9">
         <v>48</v>
       </c>
-      <c r="D73" s="12">
+      <c r="D73" s="10">
         <v>607</v>
       </c>
-      <c r="E73" s="13">
+      <c r="E73" s="11">
         <v>564</v>
       </c>
     </row>
-    <row r="74" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="10" t="s">
+    <row r="74" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A74" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="B74" s="22" t="s">
+      <c r="B74" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C74" s="11">
+      <c r="C74" s="9">
         <v>6</v>
       </c>
-      <c r="D74" s="12">
+      <c r="D74" s="10">
         <v>110</v>
       </c>
-      <c r="E74" s="13">
+      <c r="E74" s="11">
         <v>113</v>
       </c>
     </row>
-    <row r="75" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="10" t="s">
+    <row r="75" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A75" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B75" s="22" t="s">
+      <c r="B75" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C75" s="11">
+      <c r="C75" s="9">
         <v>23</v>
       </c>
-      <c r="D75" s="12">
+      <c r="D75" s="10">
         <v>161</v>
       </c>
-      <c r="E75" s="13">
+      <c r="E75" s="11">
         <v>155</v>
       </c>
     </row>
-    <row r="76" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="10" t="s">
+    <row r="76" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A76" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B76" s="22" t="s">
+      <c r="B76" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C76" s="11">
+      <c r="C76" s="9">
         <v>8</v>
       </c>
-      <c r="D76" s="12">
+      <c r="D76" s="10">
         <v>63</v>
       </c>
-      <c r="E76" s="13">
+      <c r="E76" s="11">
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="10" t="s">
+    <row r="77" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A77" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="B77" s="22" t="s">
+      <c r="B77" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C77" s="11">
+      <c r="C77" s="9">
         <v>2</v>
       </c>
-      <c r="D77" s="12">
+      <c r="D77" s="10">
         <v>39</v>
       </c>
-      <c r="E77" s="13">
+      <c r="E77" s="11">
         <v>28</v>
       </c>
     </row>
-    <row r="78" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="10" t="s">
+    <row r="78" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A78" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B78" s="22" t="s">
+      <c r="B78" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="C78" s="11">
+      <c r="C78" s="9">
         <v>9</v>
       </c>
-      <c r="D78" s="12">
+      <c r="D78" s="10">
         <v>233</v>
       </c>
-      <c r="E78" s="13">
+      <c r="E78" s="11">
         <v>193</v>
       </c>
     </row>
-    <row r="79" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="10" t="s">
+    <row r="79" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A79" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="B79" s="25" t="s">
+      <c r="B79" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="C79" s="11">
+      <c r="C79" s="9">
         <v>5</v>
       </c>
-      <c r="D79" s="12">
+      <c r="D79" s="10">
         <v>712</v>
       </c>
-      <c r="E79" s="13">
+      <c r="E79" s="11">
         <v>470</v>
       </c>
     </row>
-    <row r="80" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="10" t="s">
+    <row r="80" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A80" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="B80" s="25" t="s">
+      <c r="B80" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="C80" s="11">
+      <c r="C80" s="9">
         <v>25</v>
       </c>
-      <c r="D80" s="12">
+      <c r="D80" s="10">
         <v>378</v>
       </c>
-      <c r="E80" s="13">
+      <c r="E80" s="11">
         <v>526</v>
       </c>
     </row>
-    <row r="81" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="10" t="s">
+    <row r="81" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A81" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="B81" s="25" t="s">
+      <c r="B81" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="C81" s="11">
+      <c r="C81" s="9">
         <v>77</v>
       </c>
-      <c r="D81" s="12">
+      <c r="D81" s="10">
         <v>968</v>
       </c>
-      <c r="E81" s="13">
+      <c r="E81" s="11">
         <v>1033</v>
       </c>
     </row>
-    <row r="82" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="15" t="s">
+    <row r="82" spans="1:5" s="12" customFormat="1" ht="15" customHeight="1">
+      <c r="A82" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="B82" s="4" t="s">
+      <c r="B82" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="C82" s="16">
+      <c r="C82" s="14">
         <v>7</v>
       </c>
-      <c r="D82" s="17">
+      <c r="D82" s="15">
         <v>500</v>
       </c>
-      <c r="E82" s="18">
+      <c r="E82" s="16">
         <v>394</v>
       </c>
     </row>

</xml_diff>